<commit_message>
📊 BIST Screener | 17.04.2026 16:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-17.xlsx
+++ b/data/bist_screener_2026-04-17.xlsx
@@ -25736,40 +25736,34 @@
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B582" s="3" t="n">
-        <v>192</v>
+        <v>34.9</v>
       </c>
       <c r="C582" s="4" t="n">
-        <v>0.0549</v>
+        <v>0.0277</v>
       </c>
       <c r="D582" s="5" t="n">
-        <v>1870000</v>
-      </c>
-      <c r="E582" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>5430000</v>
+      </c>
+      <c r="E582" s="2" t="inlineStr"/>
       <c r="F582" s="3" t="n">
-        <v>83.7</v>
+        <v>61.88</v>
       </c>
       <c r="G582" s="2" t="inlineStr"/>
       <c r="H582" s="2" t="inlineStr"/>
-      <c r="I582" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J582" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I582" s="2" t="inlineStr"/>
+      <c r="J582" s="2" t="inlineStr"/>
       <c r="K582" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L582" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M582" s="2" t="inlineStr"/>
@@ -25777,56 +25771,50 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>244.9</v>
+        <v>94.25</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0.039</v>
-      </c>
-      <c r="D583" s="9" t="n">
-        <v>16940000</v>
-      </c>
+        <v>-0.048</v>
+      </c>
+      <c r="D583" s="6" t="inlineStr"/>
       <c r="E583" s="6" t="inlineStr"/>
-      <c r="F583" s="7" t="n">
-        <v>75.23999999999999</v>
-      </c>
+      <c r="F583" s="6" t="inlineStr"/>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
       <c r="I583" s="6" t="inlineStr"/>
       <c r="J583" s="6" t="inlineStr"/>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L583" s="6" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L583" s="6" t="inlineStr"/>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>6.15</v>
+        <v>4.38</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0144</v>
+        <v>0.0977</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>14310000</v>
-      </c>
-      <c r="E584" s="2" t="inlineStr"/>
+        <v>58030000</v>
+      </c>
+      <c r="E584" s="4" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F584" s="3" t="n">
-        <v>64.55</v>
+        <v>73.78</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
@@ -25837,27 +25825,33 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L584" s="2" t="inlineStr"/>
+      <c r="L584" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M584" s="2" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>24.98</v>
+        <v>261</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.0113</v>
+        <v>0.0156</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>15650000</v>
-      </c>
-      <c r="E585" s="6" t="inlineStr"/>
+        <v>9700</v>
+      </c>
+      <c r="E585" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F585" s="7" t="n">
-        <v>59.35</v>
+        <v>53.72</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
@@ -25865,75 +25859,67 @@
       <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L585" s="6" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L585" s="6" t="inlineStr"/>
       <c r="M585" s="6" t="inlineStr"/>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>6.39</v>
+        <v>7.81</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.0998</v>
+        <v>-0.08119999999999999</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>65410000</v>
+        <v>430750</v>
       </c>
       <c r="E586" s="4" t="n">
-        <v>0.1672</v>
+        <v>0.95</v>
       </c>
       <c r="F586" s="3" t="n">
-        <v>91.53</v>
+        <v>39.89</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
       <c r="I586" s="4" t="n">
-        <v>-5.3262</v>
+        <v>-23.6291</v>
       </c>
       <c r="J586" s="4" t="n">
-        <v>-4.2562</v>
+        <v>-0.4678</v>
       </c>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L586" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L586" s="2" t="inlineStr"/>
       <c r="M586" s="2" t="inlineStr"/>
     </row>
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>42.16</v>
+        <v>244.9</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0313</v>
+        <v>0.039</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>10690000</v>
+        <v>16940000</v>
       </c>
       <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>67.33</v>
+        <v>75.23999999999999</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25941,12 +25927,12 @@
       <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25954,26 +25940,34 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>34.9</v>
+        <v>17.56</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0277</v>
+        <v>0.0104</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>5430000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>13090000</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>61.88</v>
-      </c>
-      <c r="G588" s="2" t="inlineStr"/>
+        <v>50.46</v>
+      </c>
+      <c r="G588" s="3" t="n">
+        <v>165.97</v>
+      </c>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="I588" s="4" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J588" s="4" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
           <t>Üretici imalatı</t>
@@ -25981,7 +25975,7 @@
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25989,38 +25983,38 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>64.15000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0223</v>
+        <v>0.1</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>561150</v>
+        <v>228470000</v>
       </c>
       <c r="E589" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.2478</v>
       </c>
       <c r="F589" s="7" t="n">
-        <v>61.03</v>
+        <v>38.63</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="6" t="inlineStr"/>
-      <c r="J589" s="8" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="I589" s="8" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
+      <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26028,96 +26022,106 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>83.88</v>
+        <v>182.4</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0302</v>
+        <v>0.0072</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>13010000</v>
+        <v>13800000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>53.31</v>
+        <v>69.18000000000001</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="2" t="inlineStr"/>
       <c r="J590" s="2" t="inlineStr"/>
-      <c r="K590" s="2" t="inlineStr"/>
-      <c r="L590" s="2" t="inlineStr"/>
+      <c r="K590" s="2" t="inlineStr">
+        <is>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+        </is>
+      </c>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>8.140000000000001</v>
+        <v>83.7</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.1</v>
+        <v>0.034</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>228470000</v>
+        <v>34050</v>
       </c>
       <c r="E591" s="8" t="n">
-        <v>0.2478</v>
+        <v>0.58</v>
       </c>
       <c r="F591" s="7" t="n">
-        <v>38.63</v>
+        <v>43.26</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="8" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
-      <c r="J591" s="6" t="inlineStr"/>
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J591" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr"/>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>21.12</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0019</v>
-      </c>
-      <c r="D592" s="2" t="inlineStr"/>
+        <v>-0.0146</v>
+      </c>
+      <c r="D592" s="5" t="n">
+        <v>9230000</v>
+      </c>
       <c r="E592" s="2" t="inlineStr"/>
-      <c r="F592" s="2" t="inlineStr"/>
+      <c r="F592" s="3" t="n">
+        <v>77.79000000000001</v>
+      </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="2" t="inlineStr"/>
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26125,34 +26129,40 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>97.59999999999999</v>
+        <v>2.9</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0146</v>
+        <v>-0.09939999999999999</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>9230000</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>99650000</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>77.79000000000001</v>
+        <v>47.16</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J593" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26160,75 +26170,65 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>39.26</v>
+        <v>83.88</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0171</v>
+        <v>0.0302</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>13150000</v>
+        <v>13010000</v>
       </c>
       <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>51.35</v>
+        <v>53.31</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
       <c r="I594" s="2" t="inlineStr"/>
       <c r="J594" s="2" t="inlineStr"/>
-      <c r="K594" s="2" t="inlineStr">
-        <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+      <c r="K594" s="2" t="inlineStr"/>
+      <c r="L594" s="2" t="inlineStr"/>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>2.9</v>
+        <v>64.15000000000001</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.09939999999999999</v>
+        <v>0.0223</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>99650000</v>
+        <v>561150</v>
       </c>
       <c r="E595" s="8" t="n">
-        <v>0.7119</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F595" s="7" t="n">
-        <v>47.16</v>
+        <v>61.03</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
+      <c r="I595" s="6" t="inlineStr"/>
       <c r="J595" s="8" t="n">
-        <v>-0.8093</v>
+        <v>0.4139</v>
       </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26236,69 +26236,69 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>94.25</v>
+        <v>42.16</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.048</v>
-      </c>
-      <c r="D596" s="2" t="inlineStr"/>
+        <v>0.0313</v>
+      </c>
+      <c r="D596" s="5" t="n">
+        <v>10690000</v>
+      </c>
       <c r="E596" s="2" t="inlineStr"/>
-      <c r="F596" s="2" t="inlineStr"/>
+      <c r="F596" s="3" t="n">
+        <v>67.33</v>
+      </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
       <c r="I596" s="2" t="inlineStr"/>
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>17.56</v>
+        <v>3.15</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0104</v>
+        <v>0.07139999999999999</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>13090000</v>
-      </c>
-      <c r="E597" s="8" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>325930000</v>
+      </c>
+      <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>50.46</v>
-      </c>
-      <c r="G597" s="7" t="n">
-        <v>165.97</v>
-      </c>
+        <v>66.54000000000001</v>
+      </c>
+      <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J597" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I597" s="6" t="inlineStr"/>
+      <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26306,21 +26306,21 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>3.15</v>
+        <v>24.98</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.07139999999999999</v>
+        <v>0.0113</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>325930000</v>
+        <v>15650000</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>66.54000000000001</v>
+        <v>59.35</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26328,12 +26328,12 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26376,35 +26376,29 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>7.81</v>
+        <v>6.15</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.08119999999999999</v>
+        <v>-0.0144</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>430750</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>14310000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>39.89</v>
+        <v>64.55</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr"/>
@@ -26413,34 +26407,40 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>182.4</v>
+        <v>192</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0072</v>
+        <v>0.0549</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>13800000</v>
-      </c>
-      <c r="E601" s="6" t="inlineStr"/>
+        <v>1870000</v>
+      </c>
+      <c r="E601" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F601" s="7" t="n">
-        <v>69.18000000000001</v>
+        <v>83.7</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="6" t="inlineStr"/>
+      <c r="I601" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J601" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26485,71 +26485,73 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>261</v>
+        <v>21.12</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0156</v>
-      </c>
-      <c r="D603" s="9" t="n">
-        <v>9700</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.2578</v>
-      </c>
-      <c r="F603" s="7" t="n">
-        <v>53.72</v>
-      </c>
+        <v>0.0019</v>
+      </c>
+      <c r="D603" s="6" t="inlineStr"/>
+      <c r="E603" s="6" t="inlineStr"/>
+      <c r="F603" s="6" t="inlineStr"/>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
       <c r="I603" s="6" t="inlineStr"/>
       <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>83.7</v>
+        <v>6.39</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.034</v>
+        <v>0.0998</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>34050</v>
+        <v>65410000</v>
       </c>
       <c r="E604" s="4" t="n">
-        <v>0.58</v>
+        <v>0.1672</v>
       </c>
       <c r="F604" s="3" t="n">
-        <v>43.26</v>
+        <v>91.53</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
       <c r="I604" s="4" t="n">
-        <v>-9.409700000000001</v>
+        <v>-5.3262</v>
       </c>
       <c r="J604" s="4" t="n">
-        <v>-4.155</v>
+        <v>-4.2562</v>
       </c>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
@@ -26627,23 +26629,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>4.38</v>
+        <v>39.26</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0977</v>
+        <v>0.0171</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>58030000</v>
-      </c>
-      <c r="E607" s="8" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>13150000</v>
+      </c>
+      <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>73.78</v>
+        <v>51.35</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26651,12 +26651,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26683,7 +26683,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>17.04.2026 15:30</t>
+          <t>17.04.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>